<commit_message>
Finance accuracy pass: debt coverage, buyout fees and EV, paid vs blended CAC, timeline and sketch fixes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013dXhz1wBJHDaaJTjaDP8MA
</commit_message>
<xml_diff>
--- a/templates/finance-calculators.xlsx
+++ b/templates/finance-calculators.xlsx
@@ -1126,7 +1126,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Operating cash flow per year</t>
+          <t>Cash available for debt service (operating cash flow + interest paid)</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
@@ -1166,7 +1166,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Operating cash flow in a bad year</t>
+          <t>Cash available for debt service in a bad year</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
@@ -1302,11 +1302,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Cash investors put in</t>
+          <t>Cash investors put in, including deal fees</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>150000000</v>
+        <v>160000000</v>
       </c>
     </row>
     <row r="10">
@@ -1332,7 +1332,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Debt still owed at exit</t>
+          <t>Net debt at exit</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">

</xml_diff>